<commit_message>
BPMGBSA, BPSpUGBCD, BNVFE: extend file to 2070
</commit_message>
<xml_diff>
--- a/InputData/elec/BPMGBSA/BAU Policy Mandated Grid Battery Storage Additions.xlsx
+++ b/InputData/elec/BPMGBSA/BAU Policy Mandated Grid Battery Storage Additions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\BPMGBSA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\eps-mexico\InputData\elec\BPMGBSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{684B8E04-C9D8-41AD-80ED-2A9371FC7CCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C389E56-0109-4ECF-9BB5-AA5116C72F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -387,14 +387,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -413,13 +413,13 @@
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AY2"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -513,8 +513,68 @@
       <c r="AE1">
         <v>2050</v>
       </c>
+      <c r="AF1">
+        <v>2051</v>
+      </c>
+      <c r="AG1">
+        <v>2052</v>
+      </c>
+      <c r="AH1">
+        <v>2053</v>
+      </c>
+      <c r="AI1">
+        <v>2054</v>
+      </c>
+      <c r="AJ1">
+        <v>2055</v>
+      </c>
+      <c r="AK1">
+        <v>2056</v>
+      </c>
+      <c r="AL1">
+        <v>2057</v>
+      </c>
+      <c r="AM1">
+        <v>2058</v>
+      </c>
+      <c r="AN1">
+        <v>2059</v>
+      </c>
+      <c r="AO1">
+        <v>2060</v>
+      </c>
+      <c r="AP1">
+        <v>2061</v>
+      </c>
+      <c r="AQ1">
+        <v>2062</v>
+      </c>
+      <c r="AR1">
+        <v>2063</v>
+      </c>
+      <c r="AS1">
+        <v>2064</v>
+      </c>
+      <c r="AT1">
+        <v>2065</v>
+      </c>
+      <c r="AU1">
+        <v>2066</v>
+      </c>
+      <c r="AV1">
+        <v>2067</v>
+      </c>
+      <c r="AW1">
+        <v>2068</v>
+      </c>
+      <c r="AX1">
+        <v>2069</v>
+      </c>
+      <c r="AY1">
+        <v>2070</v>
+      </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.75">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -606,6 +666,66 @@
         <v>0</v>
       </c>
       <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>0</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AI2">
+        <v>0</v>
+      </c>
+      <c r="AJ2">
+        <v>0</v>
+      </c>
+      <c r="AK2">
+        <v>0</v>
+      </c>
+      <c r="AL2">
+        <v>0</v>
+      </c>
+      <c r="AM2">
+        <v>0</v>
+      </c>
+      <c r="AN2">
+        <v>0</v>
+      </c>
+      <c r="AO2">
+        <v>0</v>
+      </c>
+      <c r="AP2">
+        <v>0</v>
+      </c>
+      <c r="AQ2">
+        <v>0</v>
+      </c>
+      <c r="AR2">
+        <v>0</v>
+      </c>
+      <c r="AS2">
+        <v>0</v>
+      </c>
+      <c r="AT2">
+        <v>0</v>
+      </c>
+      <c r="AU2">
+        <v>0</v>
+      </c>
+      <c r="AV2">
+        <v>0</v>
+      </c>
+      <c r="AW2">
+        <v>0</v>
+      </c>
+      <c r="AX2">
+        <v>0</v>
+      </c>
+      <c r="AY2">
         <v>0</v>
       </c>
     </row>

</xml_diff>